<commit_message>
nRF5x QFN footprint changed bom template fixed.
</commit_message>
<xml_diff>
--- a/yildizIoT Library/Templates/BOM Supplier Links.xlsx
+++ b/yildizIoT Library/Templates/BOM Supplier Links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Common\AltiumLibrary\yildiziotlibrary\yildizIoT Library\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yldzmuhammed/Documents/Projects/altium-library/yildizIoT Library/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC4D0CE4-4C26-4F79-AA4A-FE7B1BCFBD4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5150EA5-73FE-F74A-AD03-51FA445C47B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Report" sheetId="1" r:id="rId1"/>
@@ -180,23 +180,23 @@
     <t>Column=Price</t>
   </si>
   <si>
-    <t>Column=Supplier</t>
-  </si>
-  <si>
-    <t>Column=Supplier Part Number</t>
-  </si>
-  <si>
-    <t>Column=Pricing</t>
+    <t>Column=Supplier 1</t>
+  </si>
+  <si>
+    <t>Column=Supplier Part Number 1</t>
+  </si>
+  <si>
+    <t>Column=Pricing 1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="202" formatCode="[$-C09]dd\-mmm\-yy;@"/>
-    <numFmt numFmtId="204" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="164" formatCode="[$-C09]dd\-mmm\-yy;@"/>
+    <numFmt numFmtId="165" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -206,6 +206,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -222,6 +223,7 @@
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -232,11 +234,13 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -613,10 +617,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="202" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="204" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1174,29 +1178,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" style="11" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="17.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" style="11" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="34.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="14" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A1" s="45"/>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -1210,7 +1214,7 @@
       <c r="K1" s="72"/>
       <c r="L1"/>
     </row>
-    <row r="2" spans="1:12" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="36" t="s">
         <v>40</v>
       </c>
@@ -1227,7 +1231,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="73"/>
     </row>
-    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="5" t="s">
         <v>8</v>
       </c>
@@ -1244,7 +1248,7 @@
       <c r="J3"/>
       <c r="K3" s="74"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="5" t="s">
         <v>39</v>
       </c>
@@ -1261,7 +1265,7 @@
       <c r="J4"/>
       <c r="K4" s="74"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
@@ -1278,7 +1282,7 @@
       <c r="J5"/>
       <c r="K5" s="74"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A6" s="58"/>
       <c r="B6" s="59"/>
       <c r="C6" s="29"/>
@@ -1291,7 +1295,7 @@
       <c r="J6" s="60"/>
       <c r="K6" s="75"/>
     </row>
-    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
@@ -1310,17 +1314,17 @@
       <c r="J7"/>
       <c r="K7" s="74"/>
     </row>
-    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="8">
         <f ca="1">TODAY()</f>
-        <v>45426</v>
+        <v>46142</v>
       </c>
       <c r="C8" s="9">
         <f ca="1">NOW()</f>
-        <v>45426.537888194442</v>
+        <v>46142.479913194446</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8"/>
@@ -1331,7 +1335,7 @@
       <c r="J8"/>
       <c r="K8" s="74"/>
     </row>
-    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="6"/>
       <c r="B9" s="30"/>
       <c r="C9" s="30"/>
@@ -1344,7 +1348,7 @@
       <c r="J9"/>
       <c r="K9" s="74"/>
     </row>
-    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="6" t="s">
         <v>41</v>
       </c>
@@ -1361,7 +1365,7 @@
       <c r="J10"/>
       <c r="K10" s="74"/>
     </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="6" t="s">
         <v>44</v>
       </c>
@@ -1378,7 +1382,7 @@
       <c r="J11"/>
       <c r="K11" s="74"/>
     </row>
-    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -1391,7 +1395,7 @@
       <c r="J12"/>
       <c r="K12" s="74"/>
     </row>
-    <row r="13" spans="1:12" s="35" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" s="35" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="32" t="s">
         <v>5</v>
       </c>
@@ -1426,7 +1430,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="83"/>
       <c r="B14" s="84"/>
       <c r="C14" s="83"/>
@@ -1442,7 +1446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="83"/>
       <c r="B15" s="84"/>
       <c r="C15" s="83"/>
@@ -1458,7 +1462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="83"/>
       <c r="B16" s="84"/>
       <c r="C16" s="83"/>
@@ -1474,7 +1478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A17" s="67"/>
       <c r="B17" s="68"/>
       <c r="C17" s="69"/>
@@ -1493,7 +1497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" customFormat="1" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" customFormat="1" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="48" t="s">
         <v>0</v>
       </c>
@@ -1510,7 +1514,7 @@
       <c r="J18" s="66"/>
       <c r="K18" s="76"/>
     </row>
-    <row r="19" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="51"/>
       <c r="B19" s="52"/>
       <c r="C19" s="53"/>
@@ -1523,7 +1527,7 @@
       <c r="J19" s="70"/>
       <c r="K19" s="77"/>
     </row>
-    <row r="20" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="49"/>
       <c r="B20" s="41"/>
       <c r="C20" s="42"/>
@@ -1536,7 +1540,7 @@
       <c r="J20" s="37"/>
       <c r="K20" s="78"/>
     </row>
-    <row r="21" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="49"/>
       <c r="B21" s="41"/>
       <c r="C21" s="42"/>
@@ -1549,7 +1553,7 @@
       <c r="J21" s="37"/>
       <c r="K21" s="78"/>
     </row>
-    <row r="22" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="49"/>
       <c r="B22" s="41"/>
       <c r="C22" s="42"/>
@@ -1562,7 +1566,7 @@
       <c r="J22" s="37"/>
       <c r="K22" s="78"/>
     </row>
-    <row r="23" spans="1:11" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="50"/>
       <c r="B23" s="55"/>
       <c r="C23" s="56"/>
@@ -1575,7 +1579,7 @@
       <c r="J23" s="40"/>
       <c r="K23" s="79"/>
     </row>
-    <row r="24" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="50"/>
       <c r="B24" s="39"/>
       <c r="C24" s="39"/>
@@ -1588,7 +1592,7 @@
       <c r="J24" s="40"/>
       <c r="K24" s="79"/>
     </row>
-    <row r="25" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="22"/>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -1601,7 +1605,7 @@
       <c r="J25" s="24"/>
       <c r="K25" s="80"/>
     </row>
-    <row r="26" spans="1:11" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="25"/>
       <c r="B26" s="26"/>
       <c r="C26" s="26"/>
@@ -1625,15 +1629,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" style="12" customWidth="1"/>
-    <col min="2" max="2" width="108.5703125" style="12" customWidth="1"/>
+    <col min="1" max="1" width="30.33203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="108.5" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
@@ -1641,7 +1645,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="16" t="s">
         <v>27</v>
       </c>
@@ -1649,7 +1653,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="18" t="s">
         <v>26</v>
       </c>
@@ -1657,7 +1661,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="16" t="s">
         <v>28</v>
       </c>
@@ -1665,7 +1669,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="18" t="s">
         <v>29</v>
       </c>
@@ -1673,7 +1677,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="16" t="s">
         <v>19</v>
       </c>
@@ -1681,7 +1685,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="18" t="s">
         <v>30</v>
       </c>
@@ -1689,7 +1693,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="16" t="s">
         <v>31</v>
       </c>
@@ -1697,7 +1701,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="18" t="s">
         <v>32</v>
       </c>
@@ -1705,7 +1709,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="16" t="s">
         <v>34</v>
       </c>
@@ -1713,7 +1717,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="18" t="s">
         <v>33</v>
       </c>
@@ -1721,7 +1725,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="16" t="s">
         <v>36</v>
       </c>
@@ -1729,7 +1733,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="18" t="s">
         <v>37</v>
       </c>
@@ -1737,7 +1741,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" s="15" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
         <v>38</v>
       </c>

</xml_diff>